<commit_message>
Update project period, fix the bug
</commit_message>
<xml_diff>
--- a/data/TM-RugPull_prepared_for_enrichment.xlsx
+++ b/data/TM-RugPull_prepared_for_enrichment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kseniaerofeeva/PycharmProjects/JupyterProject/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E465A57-B764-5547-A6C4-AD0BDBDF6DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1CD9DD3-CA2D-D448-B07E-96FBF58FB1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40898,7 +40898,7 @@
         <v>35</v>
       </c>
       <c r="S313" s="1">
-        <v>37455</v>
+        <v>44179</v>
       </c>
       <c r="T313" s="1">
         <v>45536</v>
@@ -43219,7 +43219,7 @@
         <v>35</v>
       </c>
       <c r="S341" s="1">
-        <v>41812</v>
+        <v>44115</v>
       </c>
       <c r="T341" s="1">
         <v>43668</v>
@@ -66113,7 +66113,7 @@
         <v>2912</v>
       </c>
       <c r="S617" s="1">
-        <v>42061</v>
+        <v>43065</v>
       </c>
       <c r="T617" s="1">
         <v>45608</v>
@@ -69018,7 +69018,7 @@
         <v>2912</v>
       </c>
       <c r="S652" s="1">
-        <v>41781</v>
+        <v>44192</v>
       </c>
       <c r="T652" s="1">
         <v>45614</v>
@@ -69101,7 +69101,7 @@
         <v>2912</v>
       </c>
       <c r="S653" s="1">
-        <v>44740</v>
+        <v>44192</v>
       </c>
       <c r="T653" s="1">
         <v>45162</v>

</xml_diff>